<commit_message>
fix: regenerate demo workbook ages to resolve to one birth date
7 of 13 patients in public/test_labs.xlsx had per-row PatientAgeAtLab
values that fit no single birth date, so the new demographics-resolution
check flagged them on first load of the shipped demo. Anchor each
patient's birth date to the midpoint of the interval implied by their
earliest row and rederive every row's age from it; only the
PatientAgeAtLab column changes, everything else round-trips untouched.

tests/fixtures/test_labs.xlsx (the parity fixture) is deliberately left
inconsistent — it exercises the conflict path and mirrors the Python
reference data.
</commit_message>
<xml_diff>
--- a/public/test_labs.xlsx
+++ b/public/test_labs.xlsx
@@ -650,7 +650,7 @@
         <v>w</v>
       </c>
       <c r="H10">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
@@ -673,7 +673,7 @@
         <v>w</v>
       </c>
       <c r="H11">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -699,7 +699,7 @@
         <v>w</v>
       </c>
       <c r="H12">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13">
@@ -725,7 +725,7 @@
         <v>w</v>
       </c>
       <c r="H13">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14">
@@ -751,7 +751,7 @@
         <v>w</v>
       </c>
       <c r="H14">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15">
@@ -777,7 +777,7 @@
         <v>w</v>
       </c>
       <c r="H15">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16">
@@ -800,7 +800,7 @@
         <v>w</v>
       </c>
       <c r="H16">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17">
@@ -823,7 +823,7 @@
         <v>w</v>
       </c>
       <c r="H17">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18">
@@ -849,7 +849,7 @@
         <v>w</v>
       </c>
       <c r="H18">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19">
@@ -875,7 +875,7 @@
         <v>w</v>
       </c>
       <c r="H19">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20">
@@ -901,7 +901,7 @@
         <v>w</v>
       </c>
       <c r="H20">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21">
@@ -927,7 +927,7 @@
         <v>w</v>
       </c>
       <c r="H21">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22">
@@ -950,7 +950,7 @@
         <v>w</v>
       </c>
       <c r="H22">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23">
@@ -976,7 +976,7 @@
         <v>w</v>
       </c>
       <c r="H23">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
@@ -1002,7 +1002,7 @@
         <v>w</v>
       </c>
       <c r="H24">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
@@ -1028,7 +1028,7 @@
         <v>w</v>
       </c>
       <c r="H25">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26">
@@ -1054,7 +1054,7 @@
         <v>w</v>
       </c>
       <c r="H26">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
@@ -1077,7 +1077,7 @@
         <v>w</v>
       </c>
       <c r="H27">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28">
@@ -1103,7 +1103,7 @@
         <v>w</v>
       </c>
       <c r="H28">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29">
@@ -1129,7 +1129,7 @@
         <v>w</v>
       </c>
       <c r="H29">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
@@ -1308,7 +1308,7 @@
         <v>m</v>
       </c>
       <c r="H36">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37">
@@ -1331,7 +1331,7 @@
         <v>m</v>
       </c>
       <c r="H37">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38">
@@ -1357,7 +1357,7 @@
         <v>m</v>
       </c>
       <c r="H38">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39">
@@ -1383,7 +1383,7 @@
         <v>m</v>
       </c>
       <c r="H39">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="40">
@@ -1409,7 +1409,7 @@
         <v>m</v>
       </c>
       <c r="H40">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="41">
@@ -1435,7 +1435,7 @@
         <v>m</v>
       </c>
       <c r="H41">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="42">
@@ -1461,7 +1461,7 @@
         <v>m</v>
       </c>
       <c r="H42">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43">
@@ -1487,7 +1487,7 @@
         <v>m</v>
       </c>
       <c r="H43">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="44">
@@ -1510,7 +1510,7 @@
         <v>m</v>
       </c>
       <c r="H44">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45">
@@ -1533,7 +1533,7 @@
         <v>m</v>
       </c>
       <c r="H45">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46">
@@ -1559,7 +1559,7 @@
         <v>m</v>
       </c>
       <c r="H46">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47">
@@ -1585,7 +1585,7 @@
         <v>m</v>
       </c>
       <c r="H47">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48">
@@ -1611,7 +1611,7 @@
         <v>m</v>
       </c>
       <c r="H48">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="49">
@@ -1637,7 +1637,7 @@
         <v>m</v>
       </c>
       <c r="H49">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50">
@@ -1660,7 +1660,7 @@
         <v>m</v>
       </c>
       <c r="H50">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51">
@@ -1683,7 +1683,7 @@
         <v>m</v>
       </c>
       <c r="H51">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="52">
@@ -1709,7 +1709,7 @@
         <v>m</v>
       </c>
       <c r="H52">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="53">
@@ -1735,7 +1735,7 @@
         <v>m</v>
       </c>
       <c r="H53">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54">
@@ -1761,7 +1761,7 @@
         <v>m</v>
       </c>
       <c r="H54">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55">
@@ -1787,7 +1787,7 @@
         <v>m</v>
       </c>
       <c r="H55">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56">
@@ -1813,7 +1813,7 @@
         <v>m</v>
       </c>
       <c r="H56">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="57">
@@ -1839,7 +1839,7 @@
         <v>m</v>
       </c>
       <c r="H57">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58">
@@ -1865,7 +1865,7 @@
         <v>m</v>
       </c>
       <c r="H58">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="59">
@@ -1891,7 +1891,7 @@
         <v>m</v>
       </c>
       <c r="H59">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="60">
@@ -1917,7 +1917,7 @@
         <v>m</v>
       </c>
       <c r="H60">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="61">
@@ -1940,7 +1940,7 @@
         <v>m</v>
       </c>
       <c r="H61">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62">
@@ -1963,7 +1963,7 @@
         <v>m</v>
       </c>
       <c r="H62">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="63">
@@ -1989,7 +1989,7 @@
         <v>m</v>
       </c>
       <c r="H63">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="64">
@@ -2015,7 +2015,7 @@
         <v>m</v>
       </c>
       <c r="H64">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65">
@@ -2041,7 +2041,7 @@
         <v>m</v>
       </c>
       <c r="H65">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66">
@@ -2067,7 +2067,7 @@
         <v>m</v>
       </c>
       <c r="H66">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="67">
@@ -2093,7 +2093,7 @@
         <v>m</v>
       </c>
       <c r="H67">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68">
@@ -2116,7 +2116,7 @@
         <v>m</v>
       </c>
       <c r="H68">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69">
@@ -2139,7 +2139,7 @@
         <v>m</v>
       </c>
       <c r="H69">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="70">
@@ -2165,7 +2165,7 @@
         <v>m</v>
       </c>
       <c r="H70">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="71">
@@ -2191,7 +2191,7 @@
         <v>m</v>
       </c>
       <c r="H71">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="72">
@@ -2321,7 +2321,7 @@
         <v>w</v>
       </c>
       <c r="H76">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77">
@@ -2347,7 +2347,7 @@
         <v>w</v>
       </c>
       <c r="H77">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="78">
@@ -2373,7 +2373,7 @@
         <v>w</v>
       </c>
       <c r="H78">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79">
@@ -2399,7 +2399,7 @@
         <v>w</v>
       </c>
       <c r="H79">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80">
@@ -2425,7 +2425,7 @@
         <v>w</v>
       </c>
       <c r="H80">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="81">
@@ -2451,7 +2451,7 @@
         <v>w</v>
       </c>
       <c r="H81">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="82">
@@ -2477,7 +2477,7 @@
         <v>w</v>
       </c>
       <c r="H82">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="83">
@@ -2500,7 +2500,7 @@
         <v>w</v>
       </c>
       <c r="H83">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="84">
@@ -2526,7 +2526,7 @@
         <v>w</v>
       </c>
       <c r="H84">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="85">
@@ -2552,7 +2552,7 @@
         <v>w</v>
       </c>
       <c r="H85">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="86">
@@ -2575,7 +2575,7 @@
         <v>w</v>
       </c>
       <c r="H86">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87">
@@ -2601,7 +2601,7 @@
         <v>w</v>
       </c>
       <c r="H87">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="88">
@@ -2624,7 +2624,7 @@
         <v>w</v>
       </c>
       <c r="H88">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="89">
@@ -2728,7 +2728,7 @@
         <v>m</v>
       </c>
       <c r="H92">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="93">
@@ -2754,7 +2754,7 @@
         <v>m</v>
       </c>
       <c r="H93">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="94">
@@ -2832,7 +2832,7 @@
         <v>m</v>
       </c>
       <c r="H96">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="97">
@@ -3016,7 +3016,7 @@
         <v>m</v>
       </c>
       <c r="H104">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="105">
@@ -3042,7 +3042,7 @@
         <v>m</v>
       </c>
       <c r="H105">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="106">
@@ -3068,7 +3068,7 @@
         <v>m</v>
       </c>
       <c r="H106">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="107">
@@ -3094,7 +3094,7 @@
         <v>m</v>
       </c>
       <c r="H107">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="108">
@@ -3120,7 +3120,7 @@
         <v>m</v>
       </c>
       <c r="H108">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="109">
@@ -3146,7 +3146,7 @@
         <v>m</v>
       </c>
       <c r="H109">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="110">
@@ -3172,7 +3172,7 @@
         <v>m</v>
       </c>
       <c r="H110">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="111">
@@ -3198,7 +3198,7 @@
         <v>m</v>
       </c>
       <c r="H111">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="112">
@@ -3354,7 +3354,7 @@
         <v>m</v>
       </c>
       <c r="H117">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="118">
@@ -3380,7 +3380,7 @@
         <v>m</v>
       </c>
       <c r="H118">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="119">
@@ -3406,7 +3406,7 @@
         <v>m</v>
       </c>
       <c r="H119">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="120">
@@ -3432,7 +3432,7 @@
         <v>m</v>
       </c>
       <c r="H120">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="121">
@@ -3458,7 +3458,7 @@
         <v>m</v>
       </c>
       <c r="H121">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="122">
@@ -3484,7 +3484,7 @@
         <v>m</v>
       </c>
       <c r="H122">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="123">
@@ -3510,7 +3510,7 @@
         <v>m</v>
       </c>
       <c r="H123">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="124">
@@ -3536,7 +3536,7 @@
         <v>m</v>
       </c>
       <c r="H124">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="125">
@@ -3562,7 +3562,7 @@
         <v>m</v>
       </c>
       <c r="H125">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="126">
@@ -3588,7 +3588,7 @@
         <v>m</v>
       </c>
       <c r="H126">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="127">
@@ -3952,7 +3952,7 @@
         <v>w</v>
       </c>
       <c r="H140">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="141">
@@ -4004,7 +4004,7 @@
         <v>w</v>
       </c>
       <c r="H142">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="143">
@@ -4030,7 +4030,7 @@
         <v>w</v>
       </c>
       <c r="H143">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="144">
@@ -4056,7 +4056,7 @@
         <v>w</v>
       </c>
       <c r="H144">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="145">
@@ -4082,7 +4082,7 @@
         <v>w</v>
       </c>
       <c r="H145">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="146">
@@ -4108,7 +4108,7 @@
         <v>w</v>
       </c>
       <c r="H146">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="147">
@@ -4134,7 +4134,7 @@
         <v>w</v>
       </c>
       <c r="H147">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="148">
@@ -4160,7 +4160,7 @@
         <v>w</v>
       </c>
       <c r="H148">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="149">
@@ -4524,7 +4524,7 @@
         <v>m</v>
       </c>
       <c r="H162">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="163">
@@ -4550,7 +4550,7 @@
         <v>m</v>
       </c>
       <c r="H163">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="164">
@@ -4784,7 +4784,7 @@
         <v>m</v>
       </c>
       <c r="H172">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="173">
@@ -4810,7 +4810,7 @@
         <v>m</v>
       </c>
       <c r="H173">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="174">
@@ -5564,7 +5564,7 @@
         <v>w</v>
       </c>
       <c r="H202">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="203">
@@ -5590,7 +5590,7 @@
         <v>w</v>
       </c>
       <c r="H203">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="204">
@@ -5668,7 +5668,7 @@
         <v>w</v>
       </c>
       <c r="H206">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="207">
@@ -5694,7 +5694,7 @@
         <v>w</v>
       </c>
       <c r="H207">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="208">
@@ -5772,7 +5772,7 @@
         <v>m</v>
       </c>
       <c r="H210">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="211">
@@ -5798,7 +5798,7 @@
         <v>m</v>
       </c>
       <c r="H211">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="212">
@@ -5928,7 +5928,7 @@
         <v>m</v>
       </c>
       <c r="H216">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="217">
@@ -5954,7 +5954,7 @@
         <v>m</v>
       </c>
       <c r="H217">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): harmonize demo workbook to multi-sheet English camelCase
</commit_message>
<xml_diff>
--- a/public/test_labs.xlsx
+++ b/public/test_labs.xlsx
@@ -1,9 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="labs" sheetId="1" r:id="rId1"/>
+    <sheet name="events" sheetId="2" r:id="rId2"/>
+    <sheet name="attributes" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -68,7 +70,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,28 +406,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>PatientID</v>
+        <v>patientId</v>
       </c>
       <c r="B1" t="str">
-        <v>LabDatum</v>
+        <v>labDate</v>
       </c>
       <c r="C1" t="str">
-        <v>Bezeichnung</v>
+        <v>testName</v>
       </c>
       <c r="D1" t="str">
-        <v>Einheit</v>
+        <v>unit</v>
       </c>
       <c r="E1" t="str">
-        <v>Wert</v>
+        <v>value</v>
       </c>
       <c r="F1" t="str">
-        <v>LOINC</v>
+        <v>loinc</v>
       </c>
       <c r="G1" t="str">
-        <v>PatientSex</v>
+        <v>sex</v>
       </c>
       <c r="H1" t="str">
-        <v>PatientAgeAtLab</v>
+        <v>ageAtLab</v>
       </c>
     </row>
     <row r="2">
@@ -5962,4 +5964,314 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H217"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>patientId</v>
+      </c>
+      <c r="B1" t="str">
+        <v>type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>date</v>
+      </c>
+      <c r="D1" t="str">
+        <v>title</v>
+      </c>
+      <c r="E1" t="str">
+        <v>intent</v>
+      </c>
+      <c r="F1" t="str">
+        <v>description</v>
+      </c>
+      <c r="G1" t="str">
+        <v>endDate</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>9</v>
+      </c>
+      <c r="B2" t="str">
+        <v>dialysis</v>
+      </c>
+      <c r="C2" s="1">
+        <v>45397</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dialysis start</v>
+      </c>
+      <c r="E2" t="str">
+        <v>chronic</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>7</v>
+      </c>
+      <c r="B3" t="str">
+        <v>dialysis</v>
+      </c>
+      <c r="C3" s="1">
+        <v>44044</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Temporary dialysis during AKI</v>
+      </c>
+      <c r="E3" t="str">
+        <v>acute</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Short acute dialysis interval in an AKI-heavy demo patient</v>
+      </c>
+      <c r="G3" s="1">
+        <v>44057</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>9</v>
+      </c>
+      <c r="B4" t="str">
+        <v>dialysis</v>
+      </c>
+      <c r="C4" s="1">
+        <v>44986</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Unknown dialysis interval</v>
+      </c>
+      <c r="E4" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Intent intentionally unknown for exclusion-policy demo</v>
+      </c>
+      <c r="G4" s="1">
+        <v>45006</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>10</v>
+      </c>
+      <c r="B5" t="str">
+        <v>kidney_transplant</v>
+      </c>
+      <c r="C5" s="1">
+        <v>45689</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Kidney transplant</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>13</v>
+      </c>
+      <c r="B6" t="str">
+        <v>kidney_transplant</v>
+      </c>
+      <c r="C6" s="1">
+        <v>44743</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Kidney transplant</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Clear pre/post transplant trajectory demo</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>14</v>
+      </c>
+      <c r="B7" t="str">
+        <v>kidney_transplant</v>
+      </c>
+      <c r="C7" s="1">
+        <v>44270</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kidney transplant</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Same-month pre/post transplant balancing demo</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>12</v>
+      </c>
+      <c r="B8" t="str">
+        <v>dialysis</v>
+      </c>
+      <c r="C8" s="1">
+        <v>45555</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Dialysis start</v>
+      </c>
+      <c r="E8" t="str">
+        <v>chronic</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>11</v>
+      </c>
+      <c r="B9" t="str">
+        <v>other</v>
+      </c>
+      <c r="C9" s="1">
+        <v>44696</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Study medication</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Display-only contextual event</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>patientId</v>
+      </c>
+      <c r="B1" t="str">
+        <v>genotype</v>
+      </c>
+      <c r="C1" t="str">
+        <v>inheritance</v>
+      </c>
+      <c r="D1" t="str">
+        <v>cohort</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>7</v>
+      </c>
+      <c r="B2" t="str">
+        <v>UMOD</v>
+      </c>
+      <c r="C2" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D2" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>8</v>
+      </c>
+      <c r="B3" t="str">
+        <v>UMOD</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D3" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>9</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MUC1</v>
+      </c>
+      <c r="C4" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D4" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>10</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PKD1</v>
+      </c>
+      <c r="C5" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D5" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>11</v>
+      </c>
+      <c r="B6" t="str">
+        <v>HNF1B</v>
+      </c>
+      <c r="C6" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D6" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>12</v>
+      </c>
+      <c r="B7" t="str">
+        <v>UMOD</v>
+      </c>
+      <c r="C7" t="str">
+        <v>AD</v>
+      </c>
+      <c r="D7" t="str">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>13</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Transplant demo</v>
+      </c>
+      <c r="D8" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>14</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Transplant demo</v>
+      </c>
+      <c r="D9" t="str">
+        <v>C</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>